<commit_message>
Update README with detailed data import instructions, including backup recommendations and import process steps. Enhance DigiKeyClient with logging for token retrieval and lookup failures. Modify Dashboard component title for clarity. Update binary files for inventory, item spread, and MPN map.
</commit_message>
<xml_diff>
--- a/phase5_1/input/inventory.xlsx
+++ b/phase5_1/input/inventory.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
   <si>
     <t>Transaction Date</t>
   </si>
@@ -72,13 +72,40 @@
     <t>DEMO-003</t>
   </si>
   <si>
-    <t>Part 863‑1523‑2‑ND</t>
-  </si>
-  <si>
     <t>DEMO-004</t>
   </si>
   <si>
-    <t>Sensor SHT40‑AD1B (1649‑…)</t>
+    <t>THERM NTC 10KOHM 3984K RING LUG</t>
+  </si>
+  <si>
+    <t>CONTACTR SS SPST-NO 35A 150-510V</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>Switching Voltage Regulators Buck Sw Reg</t>
+  </si>
+  <si>
+    <t>Circuit Breakers 508,DM,24VDC,CL,16A,ATX</t>
+  </si>
+  <si>
+    <t>584-LT1076HVIR#PBF</t>
+  </si>
+  <si>
+    <t>457-REX22DTA116E</t>
+  </si>
+  <si>
+    <t>571-10219128-02</t>
+  </si>
+  <si>
+    <t>Board Mount Temperature Sensors ESA PROBE-RTD PT1000 2000mm</t>
+  </si>
+  <si>
+    <t>225-DCM30V10L20S1PFB</t>
+  </si>
+  <si>
+    <t>Power Meters DC METER, 1000 V 300 A, ETH+RS485, MID</t>
   </si>
 </sst>
 </file>
@@ -114,9 +141,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,7 +450,7 @@
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -508,7 +534,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4">
         <v>80</v>
@@ -528,7 +554,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
         <v>19</v>
@@ -544,16 +570,96 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6">
+        <v>25</v>
+      </c>
+      <c r="F6">
+        <v>12.5</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7">
+        <v>45</v>
+      </c>
+      <c r="F7">
+        <v>45</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8">
+        <v>18</v>
+      </c>
+      <c r="F8">
+        <v>18</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9">
+        <v>120</v>
+      </c>
+      <c r="F9">
+        <v>120</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>